<commit_message>
changed text colour in shape
</commit_message>
<xml_diff>
--- a/Project/Excel/OnlineRetailDatasetSample.xlsx
+++ b/Project/Excel/OnlineRetailDatasetSample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Templates\ITVedant\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE604FBD-E563-4E8F-AEBF-164DFC6B65AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0DDE00-5ACE-448E-A230-5785E5CF79E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{796E9D62-18ED-4984-9017-94C2F0E50326}"/>
   </bookViews>
@@ -10740,13 +10740,17 @@
             <a:fld id="{AF71EEA7-F99F-47D5-AF19-F3D44ACF4994}" type="TxLink">
               <a:rPr lang="en-US" sz="2800" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
               <a:t>Total Quantity</a:t>
             </a:fld>
-            <a:endParaRPr lang="en-US" sz="2800"/>
+            <a:endParaRPr lang="en-US" sz="2800">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -10798,13 +10802,17 @@
             <a:fld id="{9489F826-3BAE-4F16-8D43-FF85D3686FEB}" type="TxLink">
               <a:rPr lang="en-US" sz="3200" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
               <a:t>3748</a:t>
             </a:fld>
-            <a:endParaRPr lang="en-US" sz="5400" b="1"/>
+            <a:endParaRPr lang="en-US" sz="5400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -10887,13 +10895,17 @@
             <a:fld id="{B41E0157-9BF5-4CA4-B2CA-82DD725DE70D}" type="TxLink">
               <a:rPr lang="en-US" sz="2800" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
               <a:t>Total Revenue</a:t>
             </a:fld>
-            <a:endParaRPr lang="en-US" sz="6000" b="1"/>
+            <a:endParaRPr lang="en-US" sz="6000" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -10945,13 +10957,17 @@
             <a:fld id="{D0A35543-88EE-45B7-AEB9-5B1DFAB10ABA}" type="TxLink">
               <a:rPr lang="en-US" sz="2800" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
               <a:t> $6,292.97 </a:t>
             </a:fld>
-            <a:endParaRPr lang="en-US" sz="11500" b="1"/>
+            <a:endParaRPr lang="en-US" sz="11500" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -11034,13 +11050,17 @@
             <a:fld id="{925C2C5E-C90A-454C-9146-F053717AFF38}" type="TxLink">
               <a:rPr lang="en-US" sz="3200" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
               <a:t>Total Transactions</a:t>
             </a:fld>
-            <a:endParaRPr lang="en-US" sz="6600" b="1"/>
+            <a:endParaRPr lang="en-US" sz="6600" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -11092,13 +11112,17 @@
             <a:fld id="{BD55BCD1-B1C8-41F2-85C5-7F806EA7E288}" type="TxLink">
               <a:rPr lang="en-US" sz="3200" b="1" i="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:schemeClr val="bg1"/>
                 </a:solidFill>
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
               <a:t>44</a:t>
             </a:fld>
-            <a:endParaRPr lang="en-US" sz="13800" b="1"/>
+            <a:endParaRPr lang="en-US" sz="13800" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>

</xml_diff>